<commit_message>
fix(quote-generate): 修复报价单模板 items 循环标记和 fallback 项目匹配
- 修复模板 {{#items}} 标记缺少闭合花括号导致循环展开失败
- 新增 _fallback_match_projects 函数，LLM 提取失败时用关键词模糊匹配项目
- attraction_search_tool 批量查询 project_table 避免 N+1
- 更新 travel-consultant 子智能体行程编排和详细行程输出规范

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/src/skills/quote-generate/templates/default.xlsx
+++ b/src/skills/quote-generate/templates/default.xlsx
@@ -5,12 +5,12 @@
   <workbookPr showInkAnnotation="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PC\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\repos\aid-work-agent\src\skills\quote-generate\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{7A0BC4F8-1CA7-45FE-AE73-A2E955622720}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA2C1844-4E77-44FC-BEBD-9D52EA0E2CCC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14475" yWindow="0" windowWidth="20310" windowHeight="18675" xr2:uid="{81ABBADA-A9A7-4DFC-83CE-445B2DB49435}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="38700" windowHeight="21900" xr2:uid="{81ABBADA-A9A7-4DFC-83CE-445B2DB49435}"/>
   </bookViews>
   <sheets>
     <sheet name="超级贵州" sheetId="3" r:id="rId1"/>
@@ -101,9 +101,6 @@
     <phoneticPr fontId="6" type="noConversion"/>
   </si>
   <si>
-    <t>{{#items}</t>
-  </si>
-  <si>
     <t>{{/items}}</t>
   </si>
   <si>
@@ -144,6 +141,10 @@
   </si>
   <si>
     <t>{{quote_per_person}}</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>{{#items}}</t>
     <phoneticPr fontId="6" type="noConversion"/>
   </si>
 </sst>
@@ -167,6 +168,7 @@
       <sz val="26"/>
       <color theme="1"/>
       <name val="宋体"/>
+      <family val="3"/>
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
@@ -175,6 +177,7 @@
       <sz val="12"/>
       <color theme="1"/>
       <name val="宋体"/>
+      <family val="3"/>
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
@@ -182,12 +185,14 @@
       <b/>
       <sz val="12"/>
       <name val="宋体"/>
+      <family val="3"/>
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="12"/>
       <name val="宋体"/>
+      <family val="3"/>
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
@@ -195,6 +200,7 @@
       <sz val="12"/>
       <color theme="1"/>
       <name val="宋体"/>
+      <family val="3"/>
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
@@ -325,17 +331,17 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="45">
+  <cellXfs count="41">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="176" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="176" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -345,12 +351,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="176" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="176" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -365,49 +365,28 @@
     <xf numFmtId="176" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="10" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="57" fontId="2" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="57" fontId="2" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -422,44 +401,59 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="176" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="57" fontId="7" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="57" fontId="7" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="57" fontId="2" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="57" fontId="2" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="10" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -775,46 +769,46 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="42" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A1" s="14" t="s">
+      <c r="A1" s="31" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="14"/>
-      <c r="C1" s="14"/>
-      <c r="D1" s="14"/>
-      <c r="E1" s="14"/>
-      <c r="F1" s="14"/>
-      <c r="G1" s="14"/>
-      <c r="H1" s="15"/>
-      <c r="I1" s="15"/>
-      <c r="J1" s="14"/>
-      <c r="K1" s="14"/>
-      <c r="L1" s="14"/>
+      <c r="B1" s="31"/>
+      <c r="C1" s="31"/>
+      <c r="D1" s="31"/>
+      <c r="E1" s="31"/>
+      <c r="F1" s="31"/>
+      <c r="G1" s="31"/>
+      <c r="H1" s="32"/>
+      <c r="I1" s="32"/>
+      <c r="J1" s="31"/>
+      <c r="K1" s="31"/>
+      <c r="L1" s="31"/>
     </row>
     <row r="2" spans="1:15" ht="39" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="34" t="s">
+      <c r="B2" s="33" t="s">
         <v>18</v>
       </c>
-      <c r="C2" s="16"/>
+      <c r="C2" s="30"/>
       <c r="D2" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="E2" s="35" t="s">
+      <c r="E2" s="34" t="s">
         <v>19</v>
       </c>
-      <c r="F2" s="17"/>
-      <c r="G2" s="17"/>
-      <c r="H2" s="17"/>
-      <c r="I2" s="18"/>
+      <c r="F2" s="35"/>
+      <c r="G2" s="35"/>
+      <c r="H2" s="35"/>
+      <c r="I2" s="36"/>
       <c r="J2" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="K2" s="36" t="s">
+      <c r="K2" s="37" t="s">
         <v>20</v>
       </c>
-      <c r="L2" s="19"/>
+      <c r="L2" s="38"/>
     </row>
     <row r="3" spans="1:15" ht="24.95" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A3" s="3" t="s">
@@ -844,67 +838,67 @@
       <c r="I3" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="J3" s="20" t="s">
+      <c r="J3" s="30" t="s">
         <v>12</v>
       </c>
-      <c r="K3" s="21"/>
-      <c r="L3" s="21"/>
-      <c r="O3" s="11"/>
+      <c r="K3" s="18"/>
+      <c r="L3" s="18"/>
+      <c r="O3" s="9"/>
     </row>
     <row r="4" spans="1:15" ht="24.95" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A4" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="B4" s="7"/>
-      <c r="C4" s="7"/>
-      <c r="D4" s="7"/>
-      <c r="E4" s="7"/>
-      <c r="F4" s="7"/>
-      <c r="G4" s="7"/>
-      <c r="H4" s="8"/>
-      <c r="I4" s="8"/>
-      <c r="J4" s="13"/>
-      <c r="K4" s="7"/>
-      <c r="L4" s="7"/>
-      <c r="O4" s="11"/>
+      <c r="A4" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="B4" s="3"/>
+      <c r="C4" s="3"/>
+      <c r="D4" s="3"/>
+      <c r="E4" s="3"/>
+      <c r="F4" s="3"/>
+      <c r="G4" s="3"/>
+      <c r="H4" s="4"/>
+      <c r="I4" s="4"/>
+      <c r="J4" s="2"/>
+      <c r="K4" s="3"/>
+      <c r="L4" s="3"/>
+      <c r="O4" s="9"/>
     </row>
     <row r="5" spans="1:15" ht="24.95" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A5" s="41" t="s">
+      <c r="A5" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="B5" s="16" t="s">
         <v>23</v>
       </c>
-      <c r="B5" s="42" t="s">
+      <c r="C5" s="16" t="s">
         <v>24</v>
       </c>
-      <c r="C5" s="42" t="s">
+      <c r="D5" s="16" t="s">
         <v>25</v>
       </c>
-      <c r="D5" s="42" t="s">
+      <c r="E5" s="16" t="s">
         <v>26</v>
       </c>
-      <c r="E5" s="42" t="s">
+      <c r="F5" s="16" t="s">
         <v>27</v>
       </c>
-      <c r="F5" s="42" t="s">
+      <c r="G5" s="16" t="s">
         <v>28</v>
       </c>
-      <c r="G5" s="42" t="s">
+      <c r="H5" s="17" t="s">
         <v>29</v>
-      </c>
-      <c r="H5" s="43" t="s">
-        <v>30</v>
       </c>
       <c r="I5" s="6">
         <v>0</v>
       </c>
-      <c r="J5" s="44" t="s">
-        <v>31</v>
-      </c>
-      <c r="K5" s="22"/>
-      <c r="L5" s="22"/>
+      <c r="J5" s="39" t="s">
+        <v>30</v>
+      </c>
+      <c r="K5" s="40"/>
+      <c r="L5" s="40"/>
     </row>
     <row r="6" spans="1:15" ht="24.95" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A6" s="37" t="s">
-        <v>22</v>
+      <c r="A6" s="11" t="s">
+        <v>21</v>
       </c>
       <c r="B6" s="5"/>
       <c r="C6" s="5"/>
@@ -913,111 +907,104 @@
       <c r="F6" s="5"/>
       <c r="G6" s="5"/>
       <c r="H6" s="6"/>
-      <c r="I6" s="12"/>
-      <c r="J6" s="38"/>
-      <c r="K6" s="39"/>
-      <c r="L6" s="40"/>
+      <c r="I6" s="10"/>
+      <c r="J6" s="12"/>
+      <c r="K6" s="13"/>
+      <c r="L6" s="14"/>
     </row>
     <row r="7" spans="1:15" ht="24.95" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A7" s="26" t="s">
+      <c r="A7" s="25" t="s">
         <v>13</v>
       </c>
-      <c r="B7" s="21"/>
-      <c r="C7" s="21"/>
-      <c r="D7" s="21"/>
-      <c r="E7" s="21"/>
-      <c r="F7" s="21"/>
-      <c r="G7" s="21"/>
-      <c r="H7" s="43" t="s">
-        <v>32</v>
-      </c>
-      <c r="I7" s="12">
+      <c r="B7" s="18"/>
+      <c r="C7" s="18"/>
+      <c r="D7" s="18"/>
+      <c r="E7" s="18"/>
+      <c r="F7" s="18"/>
+      <c r="G7" s="18"/>
+      <c r="H7" s="17" t="s">
+        <v>31</v>
+      </c>
+      <c r="I7" s="10">
         <f>SUM(I5:I5)</f>
         <v>0</v>
       </c>
-      <c r="J7" s="23"/>
-      <c r="K7" s="24"/>
-      <c r="L7" s="25"/>
+      <c r="J7" s="26"/>
+      <c r="K7" s="27"/>
+      <c r="L7" s="28"/>
     </row>
     <row r="8" spans="1:15" ht="24.95" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A8" s="21"/>
-      <c r="B8" s="21"/>
-      <c r="C8" s="21"/>
-      <c r="D8" s="21"/>
-      <c r="E8" s="21"/>
-      <c r="F8" s="21"/>
-      <c r="G8" s="21"/>
-      <c r="H8" s="27"/>
-      <c r="I8" s="27"/>
-      <c r="J8" s="20"/>
-      <c r="K8" s="21"/>
-      <c r="L8" s="21"/>
+      <c r="A8" s="18"/>
+      <c r="B8" s="18"/>
+      <c r="C8" s="18"/>
+      <c r="D8" s="18"/>
+      <c r="E8" s="18"/>
+      <c r="F8" s="18"/>
+      <c r="G8" s="18"/>
+      <c r="H8" s="29"/>
+      <c r="I8" s="29"/>
+      <c r="J8" s="30"/>
+      <c r="K8" s="18"/>
+      <c r="L8" s="18"/>
     </row>
     <row r="9" spans="1:15" ht="24.95" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A9" s="21"/>
-      <c r="B9" s="21"/>
-      <c r="C9" s="21"/>
-      <c r="D9" s="21"/>
-      <c r="E9" s="21"/>
-      <c r="F9" s="21"/>
-      <c r="G9" s="21"/>
-      <c r="H9" s="27"/>
-      <c r="I9" s="27"/>
-      <c r="J9" s="20"/>
-      <c r="K9" s="21"/>
-      <c r="L9" s="21"/>
+      <c r="A9" s="18"/>
+      <c r="B9" s="18"/>
+      <c r="C9" s="18"/>
+      <c r="D9" s="18"/>
+      <c r="E9" s="18"/>
+      <c r="F9" s="18"/>
+      <c r="G9" s="18"/>
+      <c r="H9" s="29"/>
+      <c r="I9" s="29"/>
+      <c r="J9" s="30"/>
+      <c r="K9" s="18"/>
+      <c r="L9" s="18"/>
     </row>
     <row r="10" spans="1:15" ht="24.95" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A10" s="21" t="s">
+      <c r="A10" s="18" t="s">
         <v>14</v>
       </c>
-      <c r="B10" s="28" t="s">
+      <c r="B10" s="19" t="s">
         <v>15</v>
       </c>
-      <c r="C10" s="28"/>
-      <c r="D10" s="29" t="s">
+      <c r="C10" s="19"/>
+      <c r="D10" s="20" t="s">
         <v>16</v>
       </c>
-      <c r="E10" s="29"/>
-      <c r="F10" s="29"/>
-      <c r="G10" s="29"/>
-      <c r="H10" s="30"/>
-      <c r="I10" s="9"/>
-      <c r="J10" s="31" t="s">
+      <c r="E10" s="20"/>
+      <c r="F10" s="20"/>
+      <c r="G10" s="20"/>
+      <c r="H10" s="21"/>
+      <c r="I10" s="7"/>
+      <c r="J10" s="22" t="s">
         <v>17</v>
       </c>
-      <c r="K10" s="32"/>
-      <c r="L10" s="32"/>
+      <c r="K10" s="23"/>
+      <c r="L10" s="23"/>
     </row>
     <row r="11" spans="1:15" ht="24.95" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A11" s="21"/>
-      <c r="B11" s="29" t="s">
+      <c r="A11" s="18"/>
+      <c r="B11" s="20" t="s">
         <v>2</v>
       </c>
-      <c r="C11" s="29"/>
-      <c r="D11" s="28" t="s">
+      <c r="C11" s="20"/>
+      <c r="D11" s="19" t="s">
         <v>2</v>
       </c>
-      <c r="E11" s="28"/>
-      <c r="F11" s="28"/>
-      <c r="G11" s="28"/>
-      <c r="H11" s="33"/>
-      <c r="I11" s="10"/>
-      <c r="J11" s="28" t="s">
+      <c r="E11" s="19"/>
+      <c r="F11" s="19"/>
+      <c r="G11" s="19"/>
+      <c r="H11" s="24"/>
+      <c r="I11" s="8"/>
+      <c r="J11" s="19" t="s">
         <v>2</v>
       </c>
-      <c r="K11" s="29"/>
-      <c r="L11" s="29"/>
+      <c r="K11" s="20"/>
+      <c r="L11" s="20"/>
     </row>
   </sheetData>
   <mergeCells count="17">
-    <mergeCell ref="A10:A11"/>
-    <mergeCell ref="B10:C10"/>
-    <mergeCell ref="D10:H10"/>
-    <mergeCell ref="J10:L10"/>
-    <mergeCell ref="B11:C11"/>
-    <mergeCell ref="D11:H11"/>
-    <mergeCell ref="J11:L11"/>
     <mergeCell ref="A7:G7"/>
     <mergeCell ref="J7:L7"/>
     <mergeCell ref="A8:L8"/>
@@ -1028,6 +1015,13 @@
     <mergeCell ref="K2:L2"/>
     <mergeCell ref="J3:L3"/>
     <mergeCell ref="J5:L5"/>
+    <mergeCell ref="A10:A11"/>
+    <mergeCell ref="B10:C10"/>
+    <mergeCell ref="D10:H10"/>
+    <mergeCell ref="J10:L10"/>
+    <mergeCell ref="B11:C11"/>
+    <mergeCell ref="D11:H11"/>
+    <mergeCell ref="J11:L11"/>
   </mergeCells>
   <phoneticPr fontId="6" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>